<commit_message>
Update 28 E. coli rpoB mutations with reasoning as to why they were picked.xlsx
</commit_message>
<xml_diff>
--- a/design/28 E. coli rpoB mutations with reasoning as to why they were picked.xlsx
+++ b/design/28 E. coli rpoB mutations with reasoning as to why they were picked.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janengelstaedter/Dropbox/References/_Literature Surveys/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uq-my.sharepoint.com/personal/s4844059_uq_edu_au/Documents/Documents/GitHub/RIFRxT/design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD7DF928-AB78-4287-BE49-5A27C72FE98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{AD7DF928-AB78-4287-BE49-5A27C72FE98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5334484F-613B-4680-B1C2-F83437314FDE}"/>
   <bookViews>
-    <workbookView xWindow="55240" yWindow="10120" windowWidth="21600" windowHeight="26520" firstSheet="1" activeTab="1" xr2:uid="{68D26516-A756-4642-87A8-6D8C56CEE8D1}"/>
+    <workbookView xWindow="4065" yWindow="1815" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{68D26516-A756-4642-87A8-6D8C56CEE8D1}"/>
   </bookViews>
   <sheets>
     <sheet name="overview" sheetId="1" r:id="rId1"/>
@@ -747,7 +747,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1251,7 +1251,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835599EB-1148-DD44-80E8-782CAF4AAEDB}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" style="9" customWidth="1"/>
     <col min="2" max="2" width="7.625" style="9" customWidth="1"/>
@@ -1261,7 +1261,7 @@
     <col min="6" max="16384" width="10.875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.100000000000001">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="68.099999999999994">
+    <row r="2" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="69.95" customHeight="1">
+    <row r="3" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="51">
+    <row r="4" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>13</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="51">
+    <row r="5" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="68.099999999999994">
+    <row r="6" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="68.099999999999994">
+    <row r="7" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="51">
+    <row r="8" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>27</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="51">
+    <row r="9" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>29</v>
       </c>
@@ -1413,7 +1413,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751B531C-2BD0-4376-BF32-F94025ED5114}">
   <dimension ref="A1:I30"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.625" customWidth="1"/>
     <col min="3" max="3" width="20.5" customWidth="1"/>
@@ -1425,7 +1425,7 @@
     <col min="9" max="9" width="87.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="11"/>
       <c r="B1" s="11" t="s">
         <v>32</v>
@@ -1450,7 +1450,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>39</v>
       </c>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="I2" s="10"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>45</v>
       </c>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="I3" s="10"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>48</v>
       </c>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="I4" s="10"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>51</v>
       </c>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>55</v>
       </c>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>58</v>
       </c>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>61</v>
       </c>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="I8" s="10"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>65</v>
       </c>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>68</v>
       </c>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="I10" s="10"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>71</v>
       </c>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="I11" s="10"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>74</v>
       </c>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>77</v>
       </c>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>80</v>
       </c>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>83</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>88</v>
       </c>
@@ -1795,7 +1795,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>92</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>97</v>
       </c>
@@ -1841,7 +1841,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="22" t="s">
         <v>101</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>105</v>
       </c>
@@ -1887,7 +1887,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>109</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>113</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>118</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>123</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>127</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>131</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>136</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>140</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>144</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>147</v>
       </c>
@@ -2119,7 +2119,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD11C1B-0FAA-5C4C-910E-E0951473E4DB}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.375" customWidth="1"/>
     <col min="2" max="2" width="17.125" customWidth="1"/>
@@ -2129,7 +2129,7 @@
     <col min="8" max="8" width="19.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>150</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>158</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>165</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>166</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>167</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>169</v>
       </c>
@@ -2269,13 +2269,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8029CB9A-A7C8-E24B-98A1-EE6A17216B79}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="25.625" customWidth="1"/>
     <col min="3" max="3" width="25.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>171</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>174</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>176</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>178</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>180</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>182</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>184</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>186</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>189</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>191</v>
       </c>
@@ -2396,7 +2396,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FE5F403-640D-824F-B50B-38EF5BDDF430}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="17.5" customWidth="1"/>
     <col min="5" max="5" width="13.5" customWidth="1"/>
@@ -2405,7 +2405,7 @@
     <col min="8" max="8" width="18.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>193</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>3445</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>101</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>8</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>113</v>
       </c>
@@ -2517,7 +2517,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>148</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3051</v>
       </c>
@@ -2557,7 +2557,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3595</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>3401</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>3402</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>114</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>3449</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3443</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>3370</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>111</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>7</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>3406</v>
       </c>
@@ -2819,7 +2819,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89AF531D-F3E9-7443-9620-E6682D08C81E}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="13.875" customWidth="1"/>
     <col min="5" max="5" width="19.5" customWidth="1"/>
@@ -2828,7 +2828,7 @@
     <col min="8" max="8" width="18.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>193</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>7</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>8</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
         <v>5</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>20</v>
       </c>
@@ -2949,7 +2949,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <v>22</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>23</v>
       </c>
@@ -3001,7 +3001,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>14</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>227</v>
       </c>
@@ -3086,7 +3086,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E478CBA-5B8E-8C43-A06F-FDE40A95D36E}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5" customWidth="1"/>
     <col min="2" max="2" width="50.375" customWidth="1"/>
@@ -3094,7 +3094,7 @@
     <col min="4" max="4" width="21.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>150</v>
       </c>
@@ -3108,12 +3108,12 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>231</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>187</v>
       </c>
@@ -3132,7 +3132,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>232</v>
       </c>
@@ -3158,12 +3158,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB5CB6A754A4E44785DA21A49EF665A0" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a54ed938ab0513e7a930b7d898c0a5b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f8194c36-ca64-475b-8cb3-00cec58bbf90" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6b0bb4952d1cdcfac061472cf3ae1384" ns2:_="">
     <xsd:import namespace="f8194c36-ca64-475b-8cb3-00cec58bbf90"/>
@@ -3301,14 +3295,43 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FD6D336-B253-4F96-832F-955193B4DE2D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FD6D336-B253-4F96-832F-955193B4DE2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F696F4F7-5925-4090-B9BA-CF3B9DF4C667}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D05BFA24-6847-42C9-A4B0-D3452A69DB4E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f8194c36-ca64-475b-8cb3-00cec58bbf90"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D05BFA24-6847-42C9-A4B0-D3452A69DB4E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F696F4F7-5925-4090-B9BA-CF3B9DF4C667}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>